<commit_message>
hakkurilaskentoja + ltspice tehty
</commit_message>
<xml_diff>
--- a/3teholähde_ja_jäähdytyslevy.xlsx
+++ b/3teholähde_ja_jäähdytyslevy.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
   <si>
     <t>V</t>
   </si>
@@ -27,18 +27,9 @@
     <t>U</t>
   </si>
   <si>
-    <t>f</t>
-  </si>
-  <si>
-    <t>Hz</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
-    <t>L2</t>
-  </si>
-  <si>
     <t>Henry</t>
   </si>
   <si>
@@ -70,14 +61,84 @@
   </si>
   <si>
     <t>Ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I </t>
+  </si>
+  <si>
+    <t xml:space="preserve">▲U </t>
+  </si>
+  <si>
+    <t xml:space="preserve">▲t </t>
+  </si>
+  <si>
+    <t>ohm</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>Vout</t>
+  </si>
+  <si>
+    <t>vastukset r3,r4</t>
+  </si>
+  <si>
+    <t>vastukset r1,r2</t>
+  </si>
+  <si>
+    <t>mA</t>
+  </si>
+  <si>
+    <t>C3 ja C4</t>
+  </si>
+  <si>
+    <t>ms</t>
+  </si>
+  <si>
+    <t>µF</t>
+  </si>
+  <si>
+    <t>konkat c3,c4</t>
+  </si>
+  <si>
+    <t>Hakkuri</t>
+  </si>
+  <si>
+    <t>käämit/muuntaja L2,L4</t>
+  </si>
+  <si>
+    <t>L2 ja L4</t>
+  </si>
+  <si>
+    <t>Käämi/muuntaja L1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -105,8 +166,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -128,16 +199,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>602975</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>6626</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>390526</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>57302</xdr:rowOff>
+      <xdr:colOff>75788</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>140128</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -153,8 +224,122 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3352800" y="685800"/>
-          <a:ext cx="1304926" cy="1086002"/>
+          <a:off x="3535018" y="387626"/>
+          <a:ext cx="1311552" cy="1086002"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>24848</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>165018</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>43980</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3544957" y="1739348"/>
+          <a:ext cx="1390844" cy="590632"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>49696</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>57979</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1230803</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>134376</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3594653" y="2534479"/>
+          <a:ext cx="3019846" cy="1409897"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>44246</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>143081</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3279913" y="6286500"/>
+          <a:ext cx="2495898" cy="1476581"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -429,130 +614,266 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:I13"/>
+  <dimension ref="A2:J29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
         <v>230</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="I3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>2</v>
-      </c>
-      <c r="B3">
-        <v>50</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
       </c>
       <c r="B5">
         <v>3000</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="B6">
         <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <f>(B4/B3)^2*B5</f>
+        <v>32.665406427221171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8">
+        <f>B9*B11/B10</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="2">
+        <f>0.3*10^3</f>
+        <v>300</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="2">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="2">
+        <f>0.01*10^3</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
+      <c r="C11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12">
+        <v>600</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <v>12</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="2">
+        <v>470</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="3"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="2">
+        <v>4042</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="3">
+        <v>12</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="3">
+        <f>B21/B22</f>
+        <v>40</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>230</v>
-      </c>
-      <c r="C7" t="s">
-        <v>0</v>
-      </c>
-      <c r="I7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>24</v>
-      </c>
-      <c r="C8" t="s">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <f>(B8/B7)^2*B5</f>
-        <v>32.665406427221171</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11">
-        <v>12</v>
-      </c>
-      <c r="C11" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12">
-        <v>0.3</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13">
-        <f>B11/B12</f>
-        <v>40</v>
-      </c>
-      <c r="D13" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>